<commit_message>
Initial commit for Demo 4
</commit_message>
<xml_diff>
--- a/data/FILE MẪU PHÁT THUỐC HA HẰNG NGÀY.xlsx
+++ b/data/FILE MẪU PHÁT THUỐC HA HẰNG NGÀY.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -577,7 +577,7 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>20/05/2025</v>
+        <v>21/05/2025</v>
       </c>
       <c r="J5" t="str">
         <v>I</v>
@@ -615,7 +615,7 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>20/05/2025</v>
+        <v>22/05/2025</v>
       </c>
       <c r="J6" t="str">
         <v>I</v>
@@ -653,7 +653,7 @@
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>20/05/2025</v>
+        <v>17/05/2025</v>
       </c>
       <c r="J7" t="str">
         <v>I</v>
@@ -691,7 +691,7 @@
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>20/05/2025</v>
+        <v>19/05/2025</v>
       </c>
       <c r="J8" t="str">
         <v>I</v>
@@ -767,7 +767,7 @@
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>20/05/2025</v>
+        <v>21/05/2025</v>
       </c>
       <c r="J10" t="str">
         <v>I</v>
@@ -805,7 +805,7 @@
         <v/>
       </c>
       <c r="I11" t="str">
-        <v>20/05/2025</v>
+        <v>22/05/2025</v>
       </c>
       <c r="J11" t="str">
         <v>I</v>
@@ -843,7 +843,7 @@
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>20/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J12" t="str">
         <v>I</v>
@@ -881,7 +881,7 @@
         <v/>
       </c>
       <c r="I13" t="str">
-        <v>20/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J13" t="str">
         <v>I</v>
@@ -919,7 +919,7 @@
         <v/>
       </c>
       <c r="I14" t="str">
-        <v>20/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J14" t="str">
         <v>I</v>
@@ -957,7 +957,7 @@
         <v/>
       </c>
       <c r="I15" t="str">
-        <v>20/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J15" t="str">
         <v>I</v>
@@ -995,7 +995,7 @@
         <v/>
       </c>
       <c r="I16" t="str">
-        <v>20/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J16" t="str">
         <v>I</v>
@@ -1033,7 +1033,7 @@
         <v/>
       </c>
       <c r="I17" t="str">
-        <v>20/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J17" t="str">
         <v>I</v>
@@ -1071,7 +1071,7 @@
         <v/>
       </c>
       <c r="I18" t="str">
-        <v>20/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J18" t="str">
         <v>I</v>
@@ -1109,7 +1109,7 @@
         <v/>
       </c>
       <c r="I19" t="str">
-        <v>20/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J19" t="str">
         <v>I</v>
@@ -1147,7 +1147,7 @@
         <v/>
       </c>
       <c r="I20" t="str">
-        <v>20/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J20" t="str">
         <v>I</v>
@@ -1185,7 +1185,7 @@
         <v/>
       </c>
       <c r="I21" t="str">
-        <v>20/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J21" t="str">
         <v>I</v>
@@ -1223,7 +1223,7 @@
         <v/>
       </c>
       <c r="I22" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J22" t="str">
         <v>I</v>
@@ -1261,7 +1261,7 @@
         <v/>
       </c>
       <c r="I23" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J23" t="str">
         <v>I</v>
@@ -1299,7 +1299,7 @@
         <v/>
       </c>
       <c r="I24" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J24" t="str">
         <v>I</v>
@@ -1337,7 +1337,7 @@
         <v/>
       </c>
       <c r="I25" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J25" t="str">
         <v>I</v>
@@ -1375,7 +1375,7 @@
         <v/>
       </c>
       <c r="I26" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J26" t="str">
         <v>I</v>
@@ -1413,7 +1413,7 @@
         <v/>
       </c>
       <c r="I27" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J27" t="str">
         <v>I</v>
@@ -1451,7 +1451,7 @@
         <v/>
       </c>
       <c r="I28" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J28" t="str">
         <v>I</v>
@@ -1489,7 +1489,7 @@
         <v/>
       </c>
       <c r="I29" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J29" t="str">
         <v>I</v>
@@ -1527,7 +1527,7 @@
         <v/>
       </c>
       <c r="I30" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J30" t="str">
         <v>I</v>
@@ -1565,7 +1565,7 @@
         <v/>
       </c>
       <c r="I31" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J31" t="str">
         <v>I</v>
@@ -1603,7 +1603,7 @@
         <v/>
       </c>
       <c r="I32" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J32" t="str">
         <v>I</v>
@@ -1641,7 +1641,7 @@
         <v/>
       </c>
       <c r="I33" t="str">
-        <v>20/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J33" t="str">
         <v>I</v>
@@ -1679,7 +1679,7 @@
         <v/>
       </c>
       <c r="I34" t="str">
-        <v>19/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J34" t="str">
         <v>I</v>
@@ -1717,7 +1717,7 @@
         <v/>
       </c>
       <c r="I35" t="str">
-        <v>21/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J35" t="str">
         <v>I</v>
@@ -1755,7 +1755,7 @@
         <v/>
       </c>
       <c r="I36" t="str">
-        <v>21/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J36" t="str">
         <v>I</v>
@@ -1793,7 +1793,7 @@
         <v/>
       </c>
       <c r="I37" t="str">
-        <v>21/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J37" t="str">
         <v>I</v>
@@ -1831,7 +1831,7 @@
         <v/>
       </c>
       <c r="I38" t="str">
-        <v>21/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J38" t="str">
         <v>I</v>
@@ -1869,7 +1869,7 @@
         <v/>
       </c>
       <c r="I39" t="str">
-        <v>21/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J39" t="str">
         <v>I</v>
@@ -1907,7 +1907,7 @@
         <v/>
       </c>
       <c r="I40" t="str">
-        <v>22/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J40" t="str">
         <v>I</v>
@@ -1945,7 +1945,7 @@
         <v/>
       </c>
       <c r="I41" t="str">
-        <v>21/05/2025</v>
+        <v>17/05/2025</v>
       </c>
       <c r="J41" t="str">
         <v>II</v>
@@ -1962,7 +1962,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="str">
-        <v>Trần Thiên Bình</v>
+        <v xml:space="preserve">Trần Thiên Bình </v>
       </c>
       <c r="C42">
         <v>2007</v>
@@ -1973,17 +1973,17 @@
       <c r="E42" t="str">
         <v/>
       </c>
-      <c r="F42" t="str">
+      <c r="F42">
         <v>5</v>
       </c>
       <c r="G42" t="str">
-        <v>Stanolol 50mg 1/2 v</v>
+        <v xml:space="preserve">Stanolol 50mg 1/2 v </v>
       </c>
       <c r="H42" t="str">
         <v/>
       </c>
       <c r="I42" t="str">
-        <v>29/05/2025</v>
+        <v>19/05/2025</v>
       </c>
       <c r="J42" t="str">
         <v>II</v>
@@ -2021,7 +2021,7 @@
         <v/>
       </c>
       <c r="I43" t="str">
-        <v>17/05/2025</v>
+        <v>20/05/2025</v>
       </c>
       <c r="J43" t="str">
         <v>II</v>
@@ -2059,7 +2059,7 @@
         <v/>
       </c>
       <c r="I44" t="str">
-        <v>19/05/2025</v>
+        <v>21/05/2025</v>
       </c>
       <c r="J44" t="str">
         <v>II</v>
@@ -2097,7 +2097,7 @@
         <v/>
       </c>
       <c r="I45" t="str">
-        <v>19/05/2025</v>
+        <v>22/05/2025</v>
       </c>
       <c r="J45" t="str">
         <v>II</v>
@@ -2135,7 +2135,7 @@
         <v/>
       </c>
       <c r="I46" t="str">
-        <v>19/05/2025</v>
+        <v>17/05/2025</v>
       </c>
       <c r="J46" t="str">
         <v>II</v>
@@ -2173,7 +2173,7 @@
         <v/>
       </c>
       <c r="I47" t="str">
-        <v>22/05/2025</v>
+        <v>19/05/2025</v>
       </c>
       <c r="J47" t="str">
         <v>II</v>
@@ -2211,7 +2211,7 @@
         <v/>
       </c>
       <c r="I48" t="str">
-        <v>22/05/2025</v>
+        <v>20/05/2025</v>
       </c>
       <c r="J48" t="str">
         <v>II</v>
@@ -2249,7 +2249,7 @@
         <v/>
       </c>
       <c r="I49" t="str">
-        <v>22/05/2025</v>
+        <v>21/05/2025</v>
       </c>
       <c r="J49" t="str">
         <v>II</v>
@@ -2325,7 +2325,7 @@
         <v/>
       </c>
       <c r="I51" t="str">
-        <v>22/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J51" t="str">
         <v>II</v>
@@ -2363,7 +2363,7 @@
         <v/>
       </c>
       <c r="I52" t="str">
-        <v>22/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J52" t="str">
         <v>II</v>
@@ -2401,7 +2401,7 @@
         <v/>
       </c>
       <c r="I53" t="str">
-        <v>22/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J53" t="str">
         <v>II</v>
@@ -2439,7 +2439,7 @@
         <v/>
       </c>
       <c r="I54" t="str">
-        <v>22/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J54" t="str">
         <v>II</v>
@@ -2477,7 +2477,7 @@
         <v/>
       </c>
       <c r="I55" t="str">
-        <v>22/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J55" t="str">
         <v>II</v>
@@ -2515,7 +2515,7 @@
         <v/>
       </c>
       <c r="I56" t="str">
-        <v>22/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J56" t="str">
         <v>II</v>
@@ -2553,7 +2553,7 @@
         <v/>
       </c>
       <c r="I57" t="str">
-        <v>22/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J57" t="str">
         <v>II</v>
@@ -2591,7 +2591,7 @@
         <v/>
       </c>
       <c r="I58" t="str">
-        <v>22/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J58" t="str">
         <v>II</v>
@@ -2629,7 +2629,7 @@
         <v/>
       </c>
       <c r="I59" t="str">
-        <v>22/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J59" t="str">
         <v>II</v>
@@ -2657,7 +2657,7 @@
       <c r="E60" t="str">
         <v/>
       </c>
-      <c r="F60" t="str">
+      <c r="F60">
         <v>9</v>
       </c>
       <c r="G60" t="str">
@@ -2667,7 +2667,7 @@
         <v/>
       </c>
       <c r="I60" t="str">
-        <v>28/05/2025</v>
+        <v>29/05/2025</v>
       </c>
       <c r="J60" t="str">
         <v>II</v>
@@ -2705,7 +2705,7 @@
         <v/>
       </c>
       <c r="I61" t="str">
-        <v>17/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J61" t="str">
         <v>II</v>
@@ -2743,7 +2743,7 @@
         <v/>
       </c>
       <c r="I62" t="str">
-        <v>19/05/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J62" t="str">
         <v>II</v>
@@ -2771,7 +2771,7 @@
       <c r="E63" t="str">
         <v/>
       </c>
-      <c r="F63" t="str">
+      <c r="F63">
         <v>9</v>
       </c>
       <c r="G63" t="str">
@@ -2781,10 +2781,16 @@
         <v/>
       </c>
       <c r="I63" t="str">
-        <v>03/06/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J63" t="str">
         <v>II</v>
+      </c>
+      <c r="K63" t="str">
+        <v/>
+      </c>
+      <c r="L63" t="str">
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -2810,24 +2816,56 @@
         <v>Losartan 25 mg</v>
       </c>
       <c r="H64" t="str">
-        <v>26/10/2025</v>
+        <v/>
       </c>
       <c r="I64" t="str">
-        <v>26/11/2025</v>
+        <v>30/05/2025</v>
       </c>
       <c r="J64" t="str">
+        <v>I</v>
+      </c>
+      <c r="K64" t="str">
+        <v/>
+      </c>
+      <c r="L64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="str">
+        <v>phạm quốc tâm</v>
+      </c>
+      <c r="C65">
+        <v>1987</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
+      <c r="F65" t="str">
+        <v>Nhà 2</v>
+      </c>
+      <c r="G65" t="str">
+        <v>Amlodipin 5 mg</v>
+      </c>
+      <c r="H65" t="str">
+        <v/>
+      </c>
+      <c r="I65" t="str">
+        <v>15/06/2025</v>
+      </c>
+      <c r="J65" t="str">
         <v>II</v>
-      </c>
-      <c r="K64" t="str">
-        <v/>
-      </c>
-      <c r="L64" t="str">
-        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L65"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>